<commit_message>
Complete task 2 feature selection through CV cleaning
</commit_message>
<xml_diff>
--- a/BigData/summary_reviewed.xlsx
+++ b/BigData/summary_reviewed.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="179">
   <si>
     <t xml:space="preserve">column name</t>
   </si>
@@ -682,7 +682,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3390,11 +3390,9 @@
         <v>163</v>
       </c>
       <c r="H86" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I86" s="3" t="s">
-        <v>14</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="I86" s="3"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="s">

</xml_diff>